<commit_message>
se añadio correccion de funciones y cronograma actualizado
</commit_message>
<xml_diff>
--- a/Teoria General de Sistemas/PPI/cronograma.xlsx
+++ b/Teoria General de Sistemas/PPI/cronograma.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53889F47-F0D6-4E05-9E79-D12D6AB8D399}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AFBBEAB-78ED-4B5A-ABBA-59432F85E37B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Level optizone TdeA" sheetId="11" r:id="rId1"/>
@@ -13,16 +13,28 @@
   <definedNames>
     <definedName name="hoy" localSheetId="0">TODAY()</definedName>
     <definedName name="Inicio_del_proyecto">'Level optizone TdeA'!$E$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Level optizone TdeA'!$7:$9</definedName>
     <definedName name="Semana_para_mostrar">'Level optizone TdeA'!$E$7</definedName>
     <definedName name="task_end" localSheetId="0">'Level optizone TdeA'!$F1</definedName>
     <definedName name="task_progress" localSheetId="0">'Level optizone TdeA'!$D1</definedName>
     <definedName name="task_start" localSheetId="0">'Level optizone TdeA'!$E1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Level optizone TdeA'!$7:$9</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -299,14 +311,14 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="8">
-    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0\ &quot;€&quot;_-;\-* #,##0\ &quot;€&quot;_-;_-* &quot;-&quot;\ &quot;€&quot;_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="ddd\,\ m/d/yyyy"/>
-    <numFmt numFmtId="169" formatCode="[$-C0A]d\ &quot;de&quot;\ mmmm\ &quot;de&quot;\ yyyy;@"/>
-    <numFmt numFmtId="170" formatCode="d\-m\-yy;@"/>
-    <numFmt numFmtId="171" formatCode="d"/>
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0\ &quot;€&quot;_-;\-* #,##0\ &quot;€&quot;_-;_-* &quot;-&quot;\ &quot;€&quot;_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="ddd\,\ m/d/yyyy"/>
+    <numFmt numFmtId="167" formatCode="[$-C0A]d\ &quot;de&quot;\ mmmm\ &quot;de&quot;\ yyyy;@"/>
+    <numFmt numFmtId="168" formatCode="d\-m\-yy;@"/>
+    <numFmt numFmtId="169" formatCode="d"/>
   </numFmts>
   <fonts count="33" x14ac:knownFonts="1">
     <font>
@@ -1035,7 +1047,7 @@
     </xf>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="3" applyFont="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="3" applyFont="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyProtection="0">
@@ -1044,10 +1056,10 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyProtection="0">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="3">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="3">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="2" applyFill="0">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="2" applyFill="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyFill="0">
@@ -1057,9 +1069,9 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1254,49 +1266,49 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyProtection="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="5" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="5" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="11" borderId="2" xfId="10" applyFill="1">
+    <xf numFmtId="168" fontId="9" fillId="11" borderId="2" xfId="10" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="11" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="11" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="3" borderId="2" xfId="10" applyFill="1">
+    <xf numFmtId="168" fontId="9" fillId="3" borderId="2" xfId="10" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="4" borderId="2" xfId="10" applyFill="1">
+    <xf numFmtId="168" fontId="9" fillId="4" borderId="2" xfId="10" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="10" borderId="2" xfId="10" applyFill="1">
+    <xf numFmtId="168" fontId="9" fillId="10" borderId="2" xfId="10" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="2" xfId="10">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="2" xfId="10">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1310,7 +1322,7 @@
     <xf numFmtId="9" fontId="5" fillId="45" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="46" borderId="2" xfId="12" applyFill="1">
@@ -1322,7 +1334,7 @@
     <xf numFmtId="9" fontId="5" fillId="46" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="46" borderId="2" xfId="10" applyFill="1">
+    <xf numFmtId="168" fontId="9" fillId="46" borderId="2" xfId="10" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="47" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1334,7 +1346,7 @@
     <xf numFmtId="9" fontId="5" fillId="47" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="47" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="47" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="48" borderId="2" xfId="12" applyFill="1">
@@ -1346,19 +1358,19 @@
     <xf numFmtId="9" fontId="5" fillId="48" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="48" borderId="2" xfId="10" applyFill="1">
+    <xf numFmtId="168" fontId="9" fillId="48" borderId="2" xfId="10" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8">
@@ -1367,64 +1379,64 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="3" xfId="9">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="3" xfId="9">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
-    <cellStyle name="20% - Énfasis1" xfId="31" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis2" xfId="35" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis3" xfId="39" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis4" xfId="43" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis5" xfId="47" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis6" xfId="51" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis1" xfId="32" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis2" xfId="36" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis3" xfId="40" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis4" xfId="44" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis5" xfId="48" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis6" xfId="52" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis1" xfId="33" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis2" xfId="37" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis3" xfId="41" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis4" xfId="45" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis5" xfId="49" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis6" xfId="53" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Bueno" xfId="18" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Cálculo" xfId="23" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Celda de comprobación" xfId="25" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Celda vinculada" xfId="24" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Encabezado 1" xfId="6" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Encabezado 4" xfId="17" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Énfasis1" xfId="30" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Énfasis2" xfId="34" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Énfasis3" xfId="38" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Énfasis4" xfId="42" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Énfasis5" xfId="46" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Énfasis6" xfId="50" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Entrada" xfId="21" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="31" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="35" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="39" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="43" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="47" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="51" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="32" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="36" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="40" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="44" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="48" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="52" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="33" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="37" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="41" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="45" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="49" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="53" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="30" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="34" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="38" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="42" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="46" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="50" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="19" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="23" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="25" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Comma" xfId="4" builtinId="3" customBuiltin="1"/>
+    <cellStyle name="Comma [0]" xfId="14" builtinId="6" customBuiltin="1"/>
+    <cellStyle name="Currency" xfId="15" builtinId="4" customBuiltin="1"/>
+    <cellStyle name="Currency [0]" xfId="16" builtinId="7" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="28" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Fecha" xfId="10" xr:uid="{229918B6-DD13-4F5A-97B9-305F7E002AA3}"/>
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8" customBuiltin="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="13" builtinId="9" customBuiltin="1"/>
-    <cellStyle name="Incorrecto" xfId="19" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="13" builtinId="9" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="18" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="6" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="7" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="8" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="17" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" customBuiltin="1"/>
     <cellStyle name="Inicio del proyecto" xfId="9" xr:uid="{8EB8A09A-C31C-40A3-B2C1-9449520178B8}"/>
-    <cellStyle name="Millares" xfId="4" builtinId="3" customBuiltin="1"/>
-    <cellStyle name="Millares [0]" xfId="14" builtinId="6" customBuiltin="1"/>
-    <cellStyle name="Moneda" xfId="15" builtinId="4" customBuiltin="1"/>
-    <cellStyle name="Moneda [0]" xfId="16" builtinId="7" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="21" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="24" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="20" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Nombre" xfId="11" xr:uid="{B2D3C1EE-6B41-4801-AAFC-C2274E49E503}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
-    <cellStyle name="Notas" xfId="27" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Porcentaje" xfId="2" builtinId="5" customBuiltin="1"/>
-    <cellStyle name="Salida" xfId="22" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="27" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="22" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5" customBuiltin="1"/>
     <cellStyle name="Tarea" xfId="12" xr:uid="{6391D789-272B-4DD2-9BF3-2CDCF610FA41}"/>
-    <cellStyle name="Texto de advertencia" xfId="26" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Texto explicativo" xfId="28" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Título" xfId="5" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Título 2" xfId="7" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Título 3" xfId="8" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="5" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="29" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="26" builtinId="11" customBuiltin="1"/>
     <cellStyle name="zTextoOculto" xfId="3" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
   </cellStyles>
   <dxfs count="21">
@@ -2012,21 +2024,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BS52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" style="34" customWidth="1"/>
-    <col min="2" max="2" width="51.85546875" customWidth="1"/>
+    <col min="1" max="1" width="2.6640625" style="34" customWidth="1"/>
+    <col min="2" max="2" width="51.88671875" customWidth="1"/>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" customWidth="1"/>
-    <col min="7" max="7" width="2.7109375" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" hidden="1" customWidth="1"/>
-    <col min="9" max="65" width="3.28515625" customWidth="1"/>
-    <col min="66" max="71" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" customWidth="1"/>
+    <col min="5" max="5" width="10.44140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" customWidth="1"/>
+    <col min="7" max="7" width="2.6640625" customWidth="1"/>
+    <col min="8" max="8" width="9.44140625" hidden="1" customWidth="1"/>
+    <col min="9" max="65" width="3.33203125" customWidth="1"/>
+    <col min="66" max="71" width="2.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:71" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:71" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
@@ -2040,7 +2052,7 @@
       <c r="H1" s="2"/>
       <c r="I1" s="55"/>
     </row>
-    <row r="2" spans="1:71" ht="6.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:71" ht="6.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="35"/>
       <c r="B2" s="38"/>
       <c r="C2" s="1"/>
@@ -2050,7 +2062,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="55"/>
     </row>
-    <row r="3" spans="1:71" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:71" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="34" t="s">
         <v>1</v>
       </c>
@@ -2066,7 +2078,7 @@
       <c r="I3" s="56"/>
       <c r="L3" s="72"/>
     </row>
-    <row r="4" spans="1:71" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:71" ht="18" x14ac:dyDescent="0.35">
       <c r="B4" s="73"/>
       <c r="D4" s="39" t="s">
         <v>63</v>
@@ -2077,14 +2089,14 @@
       <c r="I4" s="56"/>
       <c r="L4" s="72"/>
     </row>
-    <row r="5" spans="1:71" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:71" ht="4.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="73"/>
       <c r="D5" s="39"/>
       <c r="G5" s="39"/>
       <c r="I5" s="56"/>
       <c r="L5" s="72"/>
     </row>
-    <row r="6" spans="1:71" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:71" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="34" t="s">
         <v>2</v>
       </c>
@@ -2099,7 +2111,7 @@
       </c>
       <c r="F6" s="96"/>
     </row>
-    <row r="7" spans="1:71" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:71" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="35" t="s">
         <v>3</v>
       </c>
@@ -2109,11 +2121,11 @@
       </c>
       <c r="D7" s="95"/>
       <c r="E7" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I7" s="91">
         <f>I8</f>
-        <v>46062</v>
+        <v>46083</v>
       </c>
       <c r="J7" s="92"/>
       <c r="K7" s="92"/>
@@ -2123,7 +2135,7 @@
       <c r="O7" s="93"/>
       <c r="P7" s="91">
         <f>P8</f>
-        <v>46069</v>
+        <v>46090</v>
       </c>
       <c r="Q7" s="92"/>
       <c r="R7" s="92"/>
@@ -2133,7 +2145,7 @@
       <c r="V7" s="93"/>
       <c r="W7" s="91">
         <f>W8</f>
-        <v>46076</v>
+        <v>46097</v>
       </c>
       <c r="X7" s="92"/>
       <c r="Y7" s="92"/>
@@ -2143,7 +2155,7 @@
       <c r="AC7" s="93"/>
       <c r="AD7" s="91">
         <f>AD8</f>
-        <v>46083</v>
+        <v>46104</v>
       </c>
       <c r="AE7" s="92"/>
       <c r="AF7" s="92"/>
@@ -2153,7 +2165,7 @@
       <c r="AJ7" s="93"/>
       <c r="AK7" s="91">
         <f>AK8</f>
-        <v>46090</v>
+        <v>46111</v>
       </c>
       <c r="AL7" s="92"/>
       <c r="AM7" s="92"/>
@@ -2163,7 +2175,7 @@
       <c r="AQ7" s="93"/>
       <c r="AR7" s="91">
         <f>AR8</f>
-        <v>46097</v>
+        <v>46118</v>
       </c>
       <c r="AS7" s="92"/>
       <c r="AT7" s="92"/>
@@ -2173,7 +2185,7 @@
       <c r="AX7" s="93"/>
       <c r="AY7" s="91">
         <f>AY8</f>
-        <v>46104</v>
+        <v>46125</v>
       </c>
       <c r="AZ7" s="92"/>
       <c r="BA7" s="92"/>
@@ -2183,7 +2195,7 @@
       <c r="BE7" s="93"/>
       <c r="BF7" s="91">
         <f>BF8</f>
-        <v>46111</v>
+        <v>46132</v>
       </c>
       <c r="BG7" s="92"/>
       <c r="BH7" s="92"/>
@@ -2193,7 +2205,7 @@
       <c r="BL7" s="93"/>
       <c r="BM7" s="91">
         <f>BM8</f>
-        <v>46118</v>
+        <v>46139</v>
       </c>
       <c r="BN7" s="92"/>
       <c r="BO7" s="92"/>
@@ -2202,7 +2214,7 @@
       <c r="BR7" s="92"/>
       <c r="BS7" s="93"/>
     </row>
-    <row r="8" spans="1:71" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:71" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="35" t="s">
         <v>4</v>
       </c>
@@ -2214,258 +2226,258 @@
       <c r="G8" s="54"/>
       <c r="I8" s="65">
         <f>Inicio_del_proyecto-WEEKDAY(Inicio_del_proyecto,1)+2+7*(Semana_para_mostrar-1)</f>
-        <v>46062</v>
+        <v>46083</v>
       </c>
       <c r="J8" s="66">
         <f>I8+1</f>
-        <v>46063</v>
+        <v>46084</v>
       </c>
       <c r="K8" s="66">
         <f t="shared" ref="K8:AX8" si="0">J8+1</f>
-        <v>46064</v>
+        <v>46085</v>
       </c>
       <c r="L8" s="66">
         <f t="shared" si="0"/>
-        <v>46065</v>
+        <v>46086</v>
       </c>
       <c r="M8" s="66">
         <f t="shared" si="0"/>
-        <v>46066</v>
+        <v>46087</v>
       </c>
       <c r="N8" s="66">
         <f t="shared" si="0"/>
-        <v>46067</v>
+        <v>46088</v>
       </c>
       <c r="O8" s="67">
         <f t="shared" si="0"/>
-        <v>46068</v>
+        <v>46089</v>
       </c>
       <c r="P8" s="65">
         <f>O8+1</f>
-        <v>46069</v>
+        <v>46090</v>
       </c>
       <c r="Q8" s="66">
         <f>P8+1</f>
-        <v>46070</v>
+        <v>46091</v>
       </c>
       <c r="R8" s="66">
         <f t="shared" si="0"/>
-        <v>46071</v>
+        <v>46092</v>
       </c>
       <c r="S8" s="66">
         <f t="shared" si="0"/>
-        <v>46072</v>
+        <v>46093</v>
       </c>
       <c r="T8" s="66">
         <f t="shared" si="0"/>
-        <v>46073</v>
+        <v>46094</v>
       </c>
       <c r="U8" s="66">
         <f t="shared" si="0"/>
-        <v>46074</v>
+        <v>46095</v>
       </c>
       <c r="V8" s="67">
         <f t="shared" si="0"/>
-        <v>46075</v>
+        <v>46096</v>
       </c>
       <c r="W8" s="65">
         <f>V8+1</f>
-        <v>46076</v>
+        <v>46097</v>
       </c>
       <c r="X8" s="66">
         <f>W8+1</f>
-        <v>46077</v>
+        <v>46098</v>
       </c>
       <c r="Y8" s="66">
         <f t="shared" si="0"/>
-        <v>46078</v>
+        <v>46099</v>
       </c>
       <c r="Z8" s="66">
         <f t="shared" si="0"/>
-        <v>46079</v>
+        <v>46100</v>
       </c>
       <c r="AA8" s="66">
         <f t="shared" si="0"/>
-        <v>46080</v>
+        <v>46101</v>
       </c>
       <c r="AB8" s="66">
         <f t="shared" si="0"/>
-        <v>46081</v>
+        <v>46102</v>
       </c>
       <c r="AC8" s="67">
         <f t="shared" si="0"/>
-        <v>46082</v>
+        <v>46103</v>
       </c>
       <c r="AD8" s="65">
         <f>AC8+1</f>
-        <v>46083</v>
+        <v>46104</v>
       </c>
       <c r="AE8" s="66">
         <f>AD8+1</f>
-        <v>46084</v>
+        <v>46105</v>
       </c>
       <c r="AF8" s="66">
         <f t="shared" si="0"/>
-        <v>46085</v>
+        <v>46106</v>
       </c>
       <c r="AG8" s="66">
         <f t="shared" si="0"/>
-        <v>46086</v>
+        <v>46107</v>
       </c>
       <c r="AH8" s="66">
         <f t="shared" si="0"/>
-        <v>46087</v>
+        <v>46108</v>
       </c>
       <c r="AI8" s="66">
         <f t="shared" si="0"/>
-        <v>46088</v>
+        <v>46109</v>
       </c>
       <c r="AJ8" s="67">
         <f t="shared" si="0"/>
-        <v>46089</v>
+        <v>46110</v>
       </c>
       <c r="AK8" s="65">
         <f>AJ8+1</f>
-        <v>46090</v>
+        <v>46111</v>
       </c>
       <c r="AL8" s="66">
         <f>AK8+1</f>
-        <v>46091</v>
+        <v>46112</v>
       </c>
       <c r="AM8" s="66">
         <f t="shared" si="0"/>
-        <v>46092</v>
+        <v>46113</v>
       </c>
       <c r="AN8" s="66">
         <f t="shared" si="0"/>
-        <v>46093</v>
+        <v>46114</v>
       </c>
       <c r="AO8" s="66">
         <f t="shared" si="0"/>
-        <v>46094</v>
+        <v>46115</v>
       </c>
       <c r="AP8" s="66">
         <f t="shared" si="0"/>
-        <v>46095</v>
+        <v>46116</v>
       </c>
       <c r="AQ8" s="67">
         <f t="shared" si="0"/>
-        <v>46096</v>
+        <v>46117</v>
       </c>
       <c r="AR8" s="65">
         <f>AQ8+1</f>
-        <v>46097</v>
+        <v>46118</v>
       </c>
       <c r="AS8" s="66">
         <f>AR8+1</f>
-        <v>46098</v>
+        <v>46119</v>
       </c>
       <c r="AT8" s="66">
         <f t="shared" si="0"/>
-        <v>46099</v>
+        <v>46120</v>
       </c>
       <c r="AU8" s="66">
         <f t="shared" si="0"/>
-        <v>46100</v>
+        <v>46121</v>
       </c>
       <c r="AV8" s="66">
         <f t="shared" si="0"/>
-        <v>46101</v>
+        <v>46122</v>
       </c>
       <c r="AW8" s="66">
         <f t="shared" si="0"/>
-        <v>46102</v>
+        <v>46123</v>
       </c>
       <c r="AX8" s="67">
         <f t="shared" si="0"/>
-        <v>46103</v>
+        <v>46124</v>
       </c>
       <c r="AY8" s="65">
         <f>AX8+1</f>
-        <v>46104</v>
+        <v>46125</v>
       </c>
       <c r="AZ8" s="66">
         <f>AY8+1</f>
-        <v>46105</v>
+        <v>46126</v>
       </c>
       <c r="BA8" s="66">
         <f t="shared" ref="BA8:BE8" si="1">AZ8+1</f>
-        <v>46106</v>
+        <v>46127</v>
       </c>
       <c r="BB8" s="66">
         <f t="shared" si="1"/>
-        <v>46107</v>
+        <v>46128</v>
       </c>
       <c r="BC8" s="66">
         <f t="shared" si="1"/>
-        <v>46108</v>
+        <v>46129</v>
       </c>
       <c r="BD8" s="66">
         <f t="shared" si="1"/>
-        <v>46109</v>
+        <v>46130</v>
       </c>
       <c r="BE8" s="67">
         <f t="shared" si="1"/>
-        <v>46110</v>
+        <v>46131</v>
       </c>
       <c r="BF8" s="65">
         <f>BE8+1</f>
-        <v>46111</v>
+        <v>46132</v>
       </c>
       <c r="BG8" s="66">
         <f>BF8+1</f>
-        <v>46112</v>
+        <v>46133</v>
       </c>
       <c r="BH8" s="66">
         <f t="shared" ref="BH8:BL8" si="2">BG8+1</f>
-        <v>46113</v>
+        <v>46134</v>
       </c>
       <c r="BI8" s="66">
         <f t="shared" si="2"/>
-        <v>46114</v>
+        <v>46135</v>
       </c>
       <c r="BJ8" s="66">
         <f t="shared" si="2"/>
-        <v>46115</v>
+        <v>46136</v>
       </c>
       <c r="BK8" s="66">
         <f t="shared" si="2"/>
-        <v>46116</v>
+        <v>46137</v>
       </c>
       <c r="BL8" s="67">
         <f t="shared" si="2"/>
-        <v>46117</v>
+        <v>46138</v>
       </c>
       <c r="BM8" s="65">
         <f>BL8+1</f>
-        <v>46118</v>
+        <v>46139</v>
       </c>
       <c r="BN8" s="66">
         <f>BM8+1</f>
-        <v>46119</v>
+        <v>46140</v>
       </c>
       <c r="BO8" s="66">
         <f t="shared" ref="BO8" si="3">BN8+1</f>
-        <v>46120</v>
+        <v>46141</v>
       </c>
       <c r="BP8" s="66">
         <f t="shared" ref="BP8" si="4">BO8+1</f>
-        <v>46121</v>
+        <v>46142</v>
       </c>
       <c r="BQ8" s="66">
         <f t="shared" ref="BQ8" si="5">BP8+1</f>
-        <v>46122</v>
+        <v>46143</v>
       </c>
       <c r="BR8" s="66">
         <f t="shared" ref="BR8" si="6">BQ8+1</f>
-        <v>46123</v>
+        <v>46144</v>
       </c>
       <c r="BS8" s="67">
         <f t="shared" ref="BS8" si="7">BR8+1</f>
-        <v>46124</v>
+        <v>46145</v>
       </c>
     </row>
-    <row r="9" spans="1:71" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:71" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="35" t="s">
         <v>5</v>
       </c>
@@ -2741,7 +2753,7 @@
         <v>S</v>
       </c>
     </row>
-    <row r="10" spans="1:71" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:71" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="34" t="s">
         <v>6</v>
       </c>
@@ -2815,7 +2827,7 @@
       <c r="BR10" s="30"/>
       <c r="BS10" s="30"/>
     </row>
-    <row r="11" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="35" t="s">
         <v>7</v>
       </c>
@@ -2895,7 +2907,7 @@
       <c r="BR11" s="30"/>
       <c r="BS11" s="30"/>
     </row>
-    <row r="12" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="35" t="s">
         <v>8</v>
       </c>
@@ -2984,7 +2996,7 @@
       <c r="BR12" s="30"/>
       <c r="BS12" s="30"/>
     </row>
-    <row r="13" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="35" t="s">
         <v>9</v>
       </c>
@@ -3073,7 +3085,7 @@
       <c r="BR13" s="30"/>
       <c r="BS13" s="30"/>
     </row>
-    <row r="14" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="34"/>
       <c r="B14" s="49" t="s">
         <v>26</v>
@@ -3160,7 +3172,7 @@
       <c r="BR14" s="30"/>
       <c r="BS14" s="30"/>
     </row>
-    <row r="15" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="34"/>
       <c r="B15" s="49" t="s">
         <v>27</v>
@@ -3247,7 +3259,7 @@
       <c r="BR15" s="30"/>
       <c r="BS15" s="30"/>
     </row>
-    <row r="16" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="34"/>
       <c r="B16" s="49" t="s">
         <v>28</v>
@@ -3334,7 +3346,7 @@
       <c r="BR16" s="30"/>
       <c r="BS16" s="30"/>
     </row>
-    <row r="17" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="35" t="s">
         <v>10</v>
       </c>
@@ -3414,7 +3426,7 @@
       <c r="BR17" s="30"/>
       <c r="BS17" s="30"/>
     </row>
-    <row r="18" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="35"/>
       <c r="B18" s="50" t="s">
         <v>30</v>
@@ -3501,7 +3513,7 @@
       <c r="BR18" s="30"/>
       <c r="BS18" s="30"/>
     </row>
-    <row r="19" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="34"/>
       <c r="B19" s="50" t="s">
         <v>31</v>
@@ -3588,7 +3600,7 @@
       <c r="BR19" s="30"/>
       <c r="BS19" s="30"/>
     </row>
-    <row r="20" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="34"/>
       <c r="B20" s="50" t="s">
         <v>32</v>
@@ -3675,7 +3687,7 @@
       <c r="BR20" s="30"/>
       <c r="BS20" s="30"/>
     </row>
-    <row r="21" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="34"/>
       <c r="B21" s="50" t="s">
         <v>33</v>
@@ -3762,7 +3774,7 @@
       <c r="BR21" s="30"/>
       <c r="BS21" s="30"/>
     </row>
-    <row r="22" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="34"/>
       <c r="B22" s="50" t="s">
         <v>34</v>
@@ -3849,7 +3861,7 @@
       <c r="BR22" s="30"/>
       <c r="BS22" s="30"/>
     </row>
-    <row r="23" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="34" t="s">
         <v>11</v>
       </c>
@@ -3929,7 +3941,7 @@
       <c r="BR23" s="30"/>
       <c r="BS23" s="30"/>
     </row>
-    <row r="24" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="34"/>
       <c r="B24" s="51" t="s">
         <v>36</v>
@@ -3938,7 +3950,7 @@
         <v>58</v>
       </c>
       <c r="D24" s="22">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E24" s="62">
         <f>F24-3</f>
@@ -4016,7 +4028,7 @@
       <c r="BR24" s="30"/>
       <c r="BS24" s="30"/>
     </row>
-    <row r="25" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="34"/>
       <c r="B25" s="51" t="s">
         <v>37</v>
@@ -4025,7 +4037,7 @@
         <v>58</v>
       </c>
       <c r="D25" s="22">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E25" s="62">
         <f t="shared" ref="E25:E29" si="12">F25-3</f>
@@ -4100,7 +4112,7 @@
       <c r="BR25" s="30"/>
       <c r="BS25" s="30"/>
     </row>
-    <row r="26" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="34"/>
       <c r="B26" s="51" t="s">
         <v>38</v>
@@ -4109,7 +4121,7 @@
         <v>59</v>
       </c>
       <c r="D26" s="22">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E26" s="62">
         <f>F26-4</f>
@@ -4187,7 +4199,7 @@
       <c r="BR26" s="30"/>
       <c r="BS26" s="30"/>
     </row>
-    <row r="27" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="34"/>
       <c r="B27" s="51" t="s">
         <v>39</v>
@@ -4196,7 +4208,7 @@
         <v>55</v>
       </c>
       <c r="D27" s="22">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E27" s="62">
         <f t="shared" si="12"/>
@@ -4274,7 +4286,7 @@
       <c r="BR27" s="30"/>
       <c r="BS27" s="30"/>
     </row>
-    <row r="28" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="34"/>
       <c r="B28" s="51" t="s">
         <v>40</v>
@@ -4283,7 +4295,7 @@
         <v>66</v>
       </c>
       <c r="D28" s="22">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E28" s="62">
         <f t="shared" si="12"/>
@@ -4361,7 +4373,7 @@
       <c r="BR28" s="30"/>
       <c r="BS28" s="30"/>
     </row>
-    <row r="29" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="34"/>
       <c r="B29" s="51" t="s">
         <v>41</v>
@@ -4370,7 +4382,7 @@
         <v>56</v>
       </c>
       <c r="D29" s="22">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E29" s="62">
         <f t="shared" si="12"/>
@@ -4448,7 +4460,7 @@
       <c r="BR29" s="30"/>
       <c r="BS29" s="30"/>
     </row>
-    <row r="30" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="34" t="s">
         <v>11</v>
       </c>
@@ -4528,7 +4540,7 @@
       <c r="BR30" s="30"/>
       <c r="BS30" s="30"/>
     </row>
-    <row r="31" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="34"/>
       <c r="B31" s="52" t="s">
         <v>67</v>
@@ -4537,7 +4549,7 @@
         <v>66</v>
       </c>
       <c r="D31" s="25">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E31" s="70">
         <f>F31-2</f>
@@ -4615,7 +4627,7 @@
       <c r="BR31" s="30"/>
       <c r="BS31" s="30"/>
     </row>
-    <row r="32" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="34"/>
       <c r="B32" s="52" t="s">
         <v>68</v>
@@ -4624,7 +4636,7 @@
         <v>55</v>
       </c>
       <c r="D32" s="25">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E32" s="70">
         <f t="shared" ref="E32:E35" si="13">F32-2</f>
@@ -4702,7 +4714,7 @@
       <c r="BR32" s="30"/>
       <c r="BS32" s="30"/>
     </row>
-    <row r="33" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="34"/>
       <c r="B33" s="52" t="s">
         <v>43</v>
@@ -4711,7 +4723,7 @@
         <v>59</v>
       </c>
       <c r="D33" s="25">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E33" s="70">
         <f>F33-3</f>
@@ -4789,7 +4801,7 @@
       <c r="BR33" s="30"/>
       <c r="BS33" s="30"/>
     </row>
-    <row r="34" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="34"/>
       <c r="B34" s="52" t="s">
         <v>44</v>
@@ -4798,7 +4810,7 @@
         <v>58</v>
       </c>
       <c r="D34" s="25">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E34" s="70">
         <f t="shared" si="13"/>
@@ -4876,7 +4888,7 @@
       <c r="BR34" s="30"/>
       <c r="BS34" s="30"/>
     </row>
-    <row r="35" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="34"/>
       <c r="B35" s="52" t="s">
         <v>45</v>
@@ -4885,7 +4897,7 @@
         <v>56</v>
       </c>
       <c r="D35" s="25">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E35" s="70">
         <f t="shared" si="13"/>
@@ -4963,7 +4975,7 @@
       <c r="BR35" s="30"/>
       <c r="BS35" s="30"/>
     </row>
-    <row r="36" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="34"/>
       <c r="B36" s="74" t="s">
         <v>46</v>
@@ -5041,7 +5053,7 @@
       <c r="BR36" s="30"/>
       <c r="BS36" s="30"/>
     </row>
-    <row r="37" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="34"/>
       <c r="B37" s="78" t="s">
         <v>47</v>
@@ -5125,7 +5137,7 @@
       <c r="BR37" s="30"/>
       <c r="BS37" s="30"/>
     </row>
-    <row r="38" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="34"/>
       <c r="B38" s="78" t="s">
         <v>48</v>
@@ -5209,7 +5221,7 @@
       <c r="BR38" s="30"/>
       <c r="BS38" s="30"/>
     </row>
-    <row r="39" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="34"/>
       <c r="B39" s="78" t="s">
         <v>49</v>
@@ -5293,7 +5305,7 @@
       <c r="BR39" s="30"/>
       <c r="BS39" s="30"/>
     </row>
-    <row r="40" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="34"/>
       <c r="B40" s="78" t="s">
         <v>50</v>
@@ -5377,7 +5389,7 @@
       <c r="BR40" s="30"/>
       <c r="BS40" s="30"/>
     </row>
-    <row r="41" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="34"/>
       <c r="B41" s="78" t="s">
         <v>51</v>
@@ -5461,7 +5473,7 @@
       <c r="BR41" s="30"/>
       <c r="BS41" s="30"/>
     </row>
-    <row r="42" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="34"/>
       <c r="B42" s="82" t="s">
         <v>52</v>
@@ -5539,7 +5551,7 @@
       <c r="BR42" s="30"/>
       <c r="BS42" s="30"/>
     </row>
-    <row r="43" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="34"/>
       <c r="B43" s="86" t="s">
         <v>69</v>
@@ -5623,7 +5635,7 @@
       <c r="BR43" s="30"/>
       <c r="BS43" s="30"/>
     </row>
-    <row r="44" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="34"/>
       <c r="B44" s="86" t="s">
         <v>70</v>
@@ -5707,7 +5719,7 @@
       <c r="BR44" s="30"/>
       <c r="BS44" s="30"/>
     </row>
-    <row r="45" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="34"/>
       <c r="B45" s="86" t="s">
         <v>71</v>
@@ -5791,7 +5803,7 @@
       <c r="BR45" s="30"/>
       <c r="BS45" s="30"/>
     </row>
-    <row r="46" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="34"/>
       <c r="B46" s="86" t="s">
         <v>72</v>
@@ -5875,7 +5887,7 @@
       <c r="BR46" s="30"/>
       <c r="BS46" s="30"/>
     </row>
-    <row r="47" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="34"/>
       <c r="B47" s="86" t="s">
         <v>73</v>
@@ -5959,7 +5971,7 @@
       <c r="BR47" s="30"/>
       <c r="BS47" s="30"/>
     </row>
-    <row r="48" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="34" t="s">
         <v>12</v>
       </c>
@@ -6037,7 +6049,7 @@
       <c r="BR48" s="30"/>
       <c r="BS48" s="30"/>
     </row>
-    <row r="49" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:71" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="35" t="s">
         <v>13</v>
       </c>
@@ -6117,14 +6129,14 @@
       <c r="BR49" s="32"/>
       <c r="BS49" s="32"/>
     </row>
-    <row r="50" spans="1:71" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:71" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G50" s="6"/>
     </row>
-    <row r="51" spans="1:71" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:71" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C51" s="11"/>
       <c r="F51" s="36"/>
     </row>
-    <row r="52" spans="1:71" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:71" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C52" s="12"/>
     </row>
   </sheetData>
@@ -6360,23 +6372,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6668,29 +6669,29 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6717,9 +6718,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>